<commit_message>
Added Utility --> API,DatabaseUtility,action Methods
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Study\Selenium\workspace\OrangeHRMPageObjectModelJava\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEF5D3F-F65D-4B35-9995-790FA603A60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264234FE-5FBC-403B-ADCE-47CEAD6613FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t>username</t>
   </si>
@@ -47,10 +47,16 @@
     <t>emp_name</t>
   </si>
   <si>
-    <t>Hitendra</t>
-  </si>
-  <si>
     <t>admin</t>
+  </si>
+  <si>
+    <t>orangehrm_hverma</t>
+  </si>
+  <si>
+    <t>Passw0rd@7654321</t>
+  </si>
+  <si>
+    <t>Swapnil</t>
   </si>
 </sst>
 </file>
@@ -379,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.77734375" customWidth="1"/>
@@ -396,15 +402,24 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="Passw0rd@7654321" xr:uid="{C330EB7D-FF23-4CF1-8625-DEF5A9A5644E}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{36910CD9-610D-4757-839A-AD58D10F1E5A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -414,6 +429,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F80A6D2-5586-454F-9399-C264D9CD4478}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -454,10 +473,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates : In Excel:testdata
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Study\Selenium\workspace\OrangeHRMPageObjectModelJava\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264234FE-5FBC-403B-ADCE-47CEAD6613FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F770BA-0D8D-4ABF-B8A4-66B5F8C69A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>username</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>emp_name</t>
-  </si>
-  <si>
-    <t>admin</t>
   </si>
   <si>
     <t>orangehrm_hverma</t>
@@ -385,7 +382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.77734375" customWidth="1"/>
@@ -405,21 +402,12 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
         <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="Passw0rd@7654321" xr:uid="{C330EB7D-FF23-4CF1-8625-DEF5A9A5644E}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{36910CD9-610D-4757-839A-AD58D10F1E5A}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{36910CD9-610D-4757-839A-AD58D10F1E5A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -476,7 +464,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated test to be run on url_base
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Study\Selenium\workspace\OrangeHRMPageObjectModelJava\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F770BA-0D8D-4ABF-B8A4-66B5F8C69A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3101309-ACA8-4AD9-BCC9-F857FB6595CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>username</t>
   </si>
@@ -47,13 +47,10 @@
     <t>emp_name</t>
   </si>
   <si>
-    <t>orangehrm_hverma</t>
-  </si>
-  <si>
-    <t>Passw0rd@7654321</t>
-  </si>
-  <si>
     <t>Swapnil</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -399,15 +396,15 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{36910CD9-610D-4757-839A-AD58D10F1E5A}"/>
+    <hyperlink ref="B2" r:id="rId1" display="Passw0rd@7654321" xr:uid="{36910CD9-610D-4757-839A-AD58D10F1E5A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -464,7 +461,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>